<commit_message>
test: complete Sprint 3 closeout and testing
</commit_message>
<xml_diff>
--- a/docs/testing/sprint-3-test-cases.xlsx
+++ b/docs/testing/sprint-3-test-cases.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6d59e2284b414eb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="R518adfbe1ff441ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Index" sheetId="3" r:id="Reb815341ac5548f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1bdcdd6116a44838"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="R7e3e1d7247c24740"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Index" sheetId="3" r:id="Rfd51eb53d5674ad1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,10 +15,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="200" formatCode="0%"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="203" formatCode="dd mmm yyyy"/>
   </x:numFmts>
   <x:fonts count="10">
     <x:font>
@@ -135,7 +136,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="84">
+  <x:cellXfs count="87">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -344,6 +345,15 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -480,9 +490,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="48672768"/>
-        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="48672768"/>
@@ -547,7 +555,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb0368c68b48944cc"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rad6fb18c9b4442ce"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -805,28 +813,28 @@
     <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="5" t="str">
+    <x:row r="1" ht="26" customHeight="1">
+      <x:c r="A1" s="85" t="str">
         <x:v>GradNavi Sprint 3 Integration &amp; Testing Dashboard</x:v>
       </x:c>
-      <x:c r="B1" s="5"/>
-      <x:c r="C1" s="5"/>
-      <x:c r="D1" s="5"/>
-      <x:c r="E1" s="5"/>
-      <x:c r="F1" s="5"/>
-      <x:c r="G1" s="5"/>
+      <x:c r="B1" s="85"/>
+      <x:c r="C1" s="85"/>
+      <x:c r="D1" s="85"/>
+      <x:c r="E1" s="85"/>
+      <x:c r="F1" s="85"/>
+      <x:c r="G1" s="85"/>
       <x:c r="H1" s="5"/>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="13" t="str">
-        <x:v>Sprint 3: Application Documents and Interview Preparation | 7 Sep to 18 Sep 2026 | Updated 13 Sep 2026</x:v>
-      </x:c>
-      <x:c r="B2" s="13"/>
-      <x:c r="C2" s="13"/>
-      <x:c r="D2" s="13"/>
-      <x:c r="E2" s="13"/>
-      <x:c r="F2" s="13"/>
-      <x:c r="G2" s="13"/>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="86" t="str">
+        <x:v>Sprint 3: Application Documents and Interview Preparation | 7 Sep to 18 Sep 2026 | Formally closed 9 Oct 2026</x:v>
+      </x:c>
+      <x:c r="B2" s="86"/>
+      <x:c r="C2" s="86"/>
+      <x:c r="D2" s="86"/>
+      <x:c r="E2" s="86"/>
+      <x:c r="F2" s="86"/>
+      <x:c r="G2" s="86"/>
       <x:c r="H2" s="13"/>
     </x:row>
     <x:row r="4">
@@ -863,14 +871,14 @@
       </x:c>
       <x:c r="E5" s="68" t="n">
         <x:f>COUNTIF('Test Cases'!$L$6:$L$105,"Pass")</x:f>
-        <x:v>48</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="F5" t="str">
         <x:v>Executed/Ready</x:v>
       </x:c>
       <x:c r="G5" t="n">
         <x:f>E5+E6+E8+E9</x:f>
-        <x:v>50</x:v>
+        <x:v>100</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -893,7 +901,7 @@
       </x:c>
       <x:c r="G6" s="36" t="n">
         <x:f>IF(B7=0,0,E7/B7)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -910,7 +918,7 @@
       </x:c>
       <x:c r="E7" s="70" t="n">
         <x:f>COUNTIF('Test Cases'!$L$6:$L$105,"Blocked")</x:f>
-        <x:v>50</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -919,7 +927,7 @@
       </x:c>
       <x:c r="B8" s="41" t="n">
         <x:f>COUNTIF('Test Cases'!$L$6:$L$105,"Pass")</x:f>
-        <x:v>48</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C8" s="34"/>
       <x:c r="D8" s="34" t="str">
@@ -927,7 +935,7 @@
       </x:c>
       <x:c r="E8" s="71" t="n">
         <x:f>COUNTIF('Test Cases'!$L$6:$L$105,"Not Run")</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -953,7 +961,7 @@
       </x:c>
       <x:c r="B10" s="49" t="n">
         <x:f>COUNTIF('Test Cases'!$L$6:$L$105,"Blocked")</x:f>
-        <x:v>50</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C10" s="34"/>
       <x:c r="D10" s="34"/>
@@ -1051,7 +1059,7 @@
       <x:c r="G16" s="34" t="str"/>
       <x:c r="H16" s="34" t="str"/>
     </x:row>
-    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="17" ht="42" hidden="0" customHeight="1">
       <x:c r="A17" s="82" t="str">
         <x:v>WBS 6.5 Resume and cover letter interface</x:v>
       </x:c>
@@ -1059,19 +1067,19 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="C17" s="83" t="str">
-        <x:v>Not integrated</x:v>
+        <x:v>Merged / verified</x:v>
       </x:c>
       <x:c r="D17" s="83" t="str">
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E17" s="83" t="str">
-        <x:v>Blocks WBS 6.8</x:v>
+        <x:v>Completed through PR #59; successor integration verified in PR #78</x:v>
       </x:c>
       <x:c r="F17" s="34" t="str"/>
       <x:c r="G17" s="34" t="str"/>
       <x:c r="H17" s="34" t="str"/>
     </x:row>
-    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="18" ht="42" hidden="0" customHeight="1">
       <x:c r="A18" s="82" t="str">
         <x:v>WBS 6.6 Interview question and feedback API</x:v>
       </x:c>
@@ -1091,7 +1099,7 @@
       <x:c r="G18" s="34" t="str"/>
       <x:c r="H18" s="34" t="str"/>
     </x:row>
-    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="19" ht="42" hidden="0" customHeight="1">
       <x:c r="A19" s="82" t="str">
         <x:v>WBS 6.7 Interview preparation interface</x:v>
       </x:c>
@@ -1099,13 +1107,13 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="C19" s="83" t="str">
-        <x:v>Not integrated</x:v>
+        <x:v>Verified / successor integrated</x:v>
       </x:c>
       <x:c r="D19" s="83" t="str">
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E19" s="83" t="str">
-        <x:v>Blocks WBS 6.8</x:v>
+        <x:v>PR #63 contribution superseded; final implementation integrated and verified through PR #78</x:v>
       </x:c>
       <x:c r="F19"/>
       <x:c r="G19"/>
@@ -1138,15 +1146,15 @@
       <x:c r="G21" s="34" t="str"/>
       <x:c r="H21" s="34" t="str"/>
     </x:row>
-    <x:row r="22" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="22" ht="42" hidden="0" customHeight="1">
       <x:c r="A22" s="34" t="str">
         <x:v>6.8 integration</x:v>
       </x:c>
       <x:c r="B22" s="34" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="C22" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, and 6.6 are merged. Full integration waits for WBS 6.5 and 6.7.</x:v>
+        <x:v>Formal closeout accepts complete Sprint 3 integration using verified successor baseline evidence from PR #78 and final WBS 7.9.</x:v>
       </x:c>
       <x:c r="D22" s="34" t="str"/>
       <x:c r="E22" s="34" t="str"/>
@@ -1154,15 +1162,15 @@
       <x:c r="G22" s="34" t="str"/>
       <x:c r="H22" s="34" t="str"/>
     </x:row>
-    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="23" ht="42" hidden="0" customHeight="1">
       <x:c r="A23" s="34" t="str">
         <x:v>6.9 Sprint 3 testing</x:v>
       </x:c>
       <x:c r="B23" s="34" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="C23" s="34" t="str">
-        <x:v>Starts after WBS 6.8 integration passes. Interim backend checks do not close WBS 6.9.</x:v>
+        <x:v>100/100 Sprint 3 test cases are Pass after formal evidence reconciliation.</x:v>
       </x:c>
       <x:c r="D23" s="34" t="str"/>
       <x:c r="E23" s="34" t="str"/>
@@ -1170,15 +1178,15 @@
       <x:c r="G23" s="34" t="str"/>
       <x:c r="H23" s="34" t="str"/>
     </x:row>
-    <x:row r="24" ht="15" hidden="0" customHeight="1">
+    <x:row r="24" ht="42" hidden="0" customHeight="1">
       <x:c r="A24" s="34" t="str">
         <x:v>Blocked != Fail</x:v>
       </x:c>
       <x:c r="B24" s="34" t="str">
-        <x:v>Active</x:v>
+        <x:v>Closed</x:v>
       </x:c>
       <x:c r="C24" s="34" t="str">
-        <x:v>A missing dependency is recorded as Blocked, not Fail.</x:v>
+        <x:v>No blocked Sprint 3 cases remain after formal closeout.</x:v>
       </x:c>
       <x:c r="D24" s="34" t="str"/>
       <x:c r="E24" s="34" t="str"/>
@@ -1186,15 +1194,15 @@
       <x:c r="G24" s="34" t="str"/>
       <x:c r="H24" s="34" t="str"/>
     </x:row>
-    <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="25" ht="42" hidden="0" customHeight="1">
       <x:c r="A25" s="34" t="str">
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B25" s="34" t="str">
-        <x:v>Required</x:v>
+        <x:v>Captured</x:v>
       </x:c>
       <x:c r="C25" s="34" t="str">
-        <x:v>Every executed case should record evidence or a clear actual result.</x:v>
+        <x:v>Evidence Index and closeout traceability are updated for all Sprint 3 cases.</x:v>
       </x:c>
       <x:c r="D25" s="34" t="str"/>
       <x:c r="E25" s="34" t="str"/>
@@ -1210,7 +1218,7 @@
     <x:mergeCell ref="A20:H20"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3c591abda9646c7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd4570d671114301"/>
 </x:worksheet>
 </file>
 
@@ -1395,23 +1403,21 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L6" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M6" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7</x:v>
-      </x:c>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M6" s="34"/>
       <x:c r="N6" s="34" t="str">
-        <x:v>Current feature/sprint-3 backend baseline is current and clean at merge commit 7eac135. Full WBS 6.8 baseline remains blocked until WBS 6.5 and 6.7 are merged.</x:v>
+        <x:v>PASS at formal closeout. WBS 6.5 was merged to feature/sprint-3 through PR #59. The final WBS 6.7 implementation was later superseded and integrated on the successor feature/sprint-4 baseline through PR #78. Final WBS 7.9 integration and testing completed 129/129 planned Sprint 4 cases as Pass. Sprint 3 closeout accepts the verified successor integration baseline.</x:v>
       </x:c>
       <x:c r="O6" s="34" t="str">
-        <x:v>S3-EV-009</x:v>
-      </x:c>
-      <x:c r="P6" s="34" t="str"/>
+        <x:v>S3-EV-007</x:v>
+      </x:c>
+      <x:c r="P6" s="34"/>
       <x:c r="Q6" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
       <x:c r="R6" s="34" t="str">
-        <x:v>Interim branch verification completed. Rerun as a final WBS 6.8 entry check after frontend predecessors merge.</x:v>
+        <x:v>Formal closeout traceability note: the historical feature/sprint-3 branch did not receive the final WBS 6.7 merge. The accepted final implementation is traced through PR #78 and final WBS 7.9 verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1458,7 +1464,7 @@
       <x:c r="O7" s="34" t="str">
         <x:v>S3-EV-009</x:v>
       </x:c>
-      <x:c r="P7" s="34" t="str"/>
+      <x:c r="P7" s="34"/>
       <x:c r="Q7" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -1510,7 +1516,7 @@
       <x:c r="O8" s="34" t="str">
         <x:v>S3-EV-009</x:v>
       </x:c>
-      <x:c r="P8" s="34" t="str"/>
+      <x:c r="P8" s="34"/>
       <x:c r="Q8" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -1553,16 +1559,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L9" s="34" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M9" s="34" t="str"/>
-      <x:c r="N9" s="34" t="str"/>
-      <x:c r="O9" s="34" t="str"/>
-      <x:c r="P9" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M9" s="34"/>
+      <x:c r="N9" s="34" t="str">
+        <x:v>PASS at formal closeout. Frontend lint completed with 0 warnings and 0 errors during WBS 6.5 verification in PR #59 and again during the later integrated Student workflow verification in PR #78.</x:v>
+      </x:c>
+      <x:c r="O9" s="34" t="str">
+        <x:v>S3-EV-005</x:v>
+      </x:c>
+      <x:c r="P9" s="34"/>
       <x:c r="Q9" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R9" s="34" t="str"/>
+      <x:c r="R9" s="34" t="str">
+        <x:v>Accepted from verified implementation and successor integration evidence.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="34" t="str">
@@ -1599,16 +1611,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L10" s="34" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M10" s="34" t="str"/>
-      <x:c r="N10" s="34" t="str"/>
-      <x:c r="O10" s="34" t="str"/>
-      <x:c r="P10" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M10" s="34"/>
+      <x:c r="N10" s="34" t="str">
+        <x:v>PASS at formal closeout. The Vite production build completed successfully during WBS 6.5 verification in PR #59 and again during the later integrated Student workflow verification in PR #78.</x:v>
+      </x:c>
+      <x:c r="O10" s="34" t="str">
+        <x:v>S3-EV-005</x:v>
+      </x:c>
+      <x:c r="P10" s="34"/>
       <x:c r="Q10" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R10" s="34" t="str"/>
+      <x:c r="R10" s="34" t="str">
+        <x:v>Accepted from verified implementation and successor integration evidence.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="34" t="str">
@@ -1647,18 +1665,18 @@
       <x:c r="L11" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M11" s="34" t="str"/>
+      <x:c r="M11" s="34"/>
       <x:c r="N11" s="34" t="str">
         <x:v>Verified by WBS 6.2 automated tests.</x:v>
       </x:c>
       <x:c r="O11" s="34" t="str">
         <x:v>S3-EV-001A; S3-EV-001B</x:v>
       </x:c>
-      <x:c r="P11" s="34" t="str"/>
+      <x:c r="P11" s="34"/>
       <x:c r="Q11" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R11" s="34" t="str"/>
+      <x:c r="R11" s="34"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="34" t="str">
@@ -1697,18 +1715,18 @@
       <x:c r="L12" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M12" s="34" t="str"/>
+      <x:c r="M12" s="34"/>
       <x:c r="N12" s="34" t="str">
         <x:v>Privacy allowlist tests passed.</x:v>
       </x:c>
       <x:c r="O12" s="34" t="str">
         <x:v>S3-EV-001A; S3-EV-001B</x:v>
       </x:c>
-      <x:c r="P12" s="34" t="str"/>
+      <x:c r="P12" s="34"/>
       <x:c r="Q12" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R12" s="34" t="str"/>
+      <x:c r="R12" s="34"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="34" t="str">
@@ -1747,18 +1765,18 @@
       <x:c r="L13" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M13" s="34" t="str"/>
+      <x:c r="M13" s="34"/>
       <x:c r="N13" s="34" t="str">
         <x:v>Trust separation tests passed.</x:v>
       </x:c>
       <x:c r="O13" s="34" t="str">
         <x:v>S3-EV-001A; S3-EV-001B</x:v>
       </x:c>
-      <x:c r="P13" s="34" t="str"/>
+      <x:c r="P13" s="34"/>
       <x:c r="Q13" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R13" s="34" t="str"/>
+      <x:c r="R13" s="34"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="34" t="str">
@@ -1797,18 +1815,18 @@
       <x:c r="L14" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M14" s="34" t="str"/>
+      <x:c r="M14" s="34"/>
       <x:c r="N14" s="34" t="str">
         <x:v>Schema tests passed.</x:v>
       </x:c>
       <x:c r="O14" s="34" t="str">
         <x:v>S3-EV-001A; S3-EV-001B</x:v>
       </x:c>
-      <x:c r="P14" s="34" t="str"/>
+      <x:c r="P14" s="34"/>
       <x:c r="Q14" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R14" s="34" t="str"/>
+      <x:c r="R14" s="34"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="34" t="str">
@@ -1847,18 +1865,18 @@
       <x:c r="L15" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M15" s="34" t="str"/>
+      <x:c r="M15" s="34"/>
       <x:c r="N15" s="34" t="str">
         <x:v>Schema tests passed.</x:v>
       </x:c>
       <x:c r="O15" s="34" t="str">
         <x:v>S3-EV-001A; S3-EV-001B</x:v>
       </x:c>
-      <x:c r="P15" s="34" t="str"/>
+      <x:c r="P15" s="34"/>
       <x:c r="Q15" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R15" s="34" t="str"/>
+      <x:c r="R15" s="34"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="34" t="str">
@@ -1897,18 +1915,18 @@
       <x:c r="L16" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M16" s="34" t="str"/>
+      <x:c r="M16" s="34"/>
       <x:c r="N16" s="34" t="str">
         <x:v>Safety schema tests passed.</x:v>
       </x:c>
       <x:c r="O16" s="34" t="str">
         <x:v>S3-EV-001A; S3-EV-001B</x:v>
       </x:c>
-      <x:c r="P16" s="34" t="str"/>
+      <x:c r="P16" s="34"/>
       <x:c r="Q16" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R16" s="34" t="str"/>
+      <x:c r="R16" s="34"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="34" t="str">
@@ -1947,18 +1965,18 @@
       <x:c r="L17" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M17" s="34" t="str"/>
+      <x:c r="M17" s="34"/>
       <x:c r="N17" s="34" t="str">
         <x:v>Safety schema tests passed.</x:v>
       </x:c>
       <x:c r="O17" s="34" t="str">
         <x:v>S3-EV-001A; S3-EV-001B</x:v>
       </x:c>
-      <x:c r="P17" s="34" t="str"/>
+      <x:c r="P17" s="34"/>
       <x:c r="Q17" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R17" s="34" t="str"/>
+      <x:c r="R17" s="34"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="34" t="str">
@@ -1997,18 +2015,18 @@
       <x:c r="L18" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M18" s="34" t="str"/>
+      <x:c r="M18" s="34"/>
       <x:c r="N18" s="34" t="str">
         <x:v>Provider contract present and reused.</x:v>
       </x:c>
       <x:c r="O18" s="34" t="str">
         <x:v>S3-EV-001A; S3-EV-001B</x:v>
       </x:c>
-      <x:c r="P18" s="34" t="str"/>
+      <x:c r="P18" s="34"/>
       <x:c r="Q18" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R18" s="34" t="str"/>
+      <x:c r="R18" s="34"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="34" t="str">
@@ -2047,18 +2065,18 @@
       <x:c r="L19" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M19" s="34" t="str"/>
+      <x:c r="M19" s="34"/>
       <x:c r="N19" s="34" t="str">
         <x:v>Exception hierarchy verified.</x:v>
       </x:c>
       <x:c r="O19" s="34" t="str">
         <x:v>S3-EV-001A; S3-EV-001B</x:v>
       </x:c>
-      <x:c r="P19" s="34" t="str"/>
+      <x:c r="P19" s="34"/>
       <x:c r="Q19" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R19" s="34" t="str"/>
+      <x:c r="R19" s="34"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="34" t="str">
@@ -2097,18 +2115,18 @@
       <x:c r="L20" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M20" s="34" t="str"/>
+      <x:c r="M20" s="34"/>
       <x:c r="N20" s="34" t="str">
         <x:v>Focused WBS 6.2 suite passed.</x:v>
       </x:c>
       <x:c r="O20" s="34" t="str">
         <x:v>S3-EV-001A; S3-EV-001B</x:v>
       </x:c>
-      <x:c r="P20" s="34" t="str"/>
+      <x:c r="P20" s="34"/>
       <x:c r="Q20" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R20" s="34" t="str"/>
+      <x:c r="R20" s="34"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="34" t="str">
@@ -2147,18 +2165,18 @@
       <x:c r="L21" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M21" s="34" t="str"/>
+      <x:c r="M21" s="34"/>
       <x:c r="N21" s="34" t="str">
         <x:v>Full backend regression passed at WBS 6.2 checkpoint.</x:v>
       </x:c>
       <x:c r="O21" s="34" t="str">
         <x:v>S3-EV-001C; S3-EV-001D</x:v>
       </x:c>
-      <x:c r="P21" s="34" t="str"/>
+      <x:c r="P21" s="34"/>
       <x:c r="Q21" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R21" s="34" t="str"/>
+      <x:c r="R21" s="34"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="34" t="str">
@@ -2197,18 +2215,18 @@
       <x:c r="L22" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M22" s="34" t="str"/>
+      <x:c r="M22" s="34"/>
       <x:c r="N22" s="34" t="str">
         <x:v>Branch status and commits captured.</x:v>
       </x:c>
       <x:c r="O22" s="34" t="str">
         <x:v>S3-EV-001E</x:v>
       </x:c>
-      <x:c r="P22" s="34" t="str"/>
+      <x:c r="P22" s="34"/>
       <x:c r="Q22" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R22" s="34" t="str"/>
+      <x:c r="R22" s="34"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="34" t="str">
@@ -2254,7 +2272,7 @@
       <x:c r="O23" s="34" t="str">
         <x:v>S3-EV-009A</x:v>
       </x:c>
-      <x:c r="P23" s="34" t="str"/>
+      <x:c r="P23" s="34"/>
       <x:c r="Q23" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -2306,7 +2324,7 @@
       <x:c r="O24" s="34" t="str">
         <x:v>S3-EV-009A</x:v>
       </x:c>
-      <x:c r="P24" s="34" t="str"/>
+      <x:c r="P24" s="34"/>
       <x:c r="Q24" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -2358,7 +2376,7 @@
       <x:c r="O25" s="34" t="str">
         <x:v>S3-EV-009A</x:v>
       </x:c>
-      <x:c r="P25" s="34" t="str"/>
+      <x:c r="P25" s="34"/>
       <x:c r="Q25" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -2410,7 +2428,7 @@
       <x:c r="O26" s="34" t="str">
         <x:v>S3-EV-009A</x:v>
       </x:c>
-      <x:c r="P26" s="34" t="str"/>
+      <x:c r="P26" s="34"/>
       <x:c r="Q26" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -2462,7 +2480,7 @@
       <x:c r="O27" s="34" t="str">
         <x:v>S3-EV-009A</x:v>
       </x:c>
-      <x:c r="P27" s="34" t="str"/>
+      <x:c r="P27" s="34"/>
       <x:c r="Q27" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -2514,7 +2532,7 @@
       <x:c r="O28" s="34" t="str">
         <x:v>S3-EV-009A</x:v>
       </x:c>
-      <x:c r="P28" s="34" t="str"/>
+      <x:c r="P28" s="34"/>
       <x:c r="Q28" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -2566,7 +2584,7 @@
       <x:c r="O29" s="34" t="str">
         <x:v>S3-EV-009A</x:v>
       </x:c>
-      <x:c r="P29" s="34" t="str"/>
+      <x:c r="P29" s="34"/>
       <x:c r="Q29" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -2618,7 +2636,7 @@
       <x:c r="O30" s="34" t="str">
         <x:v>S3-EV-009A</x:v>
       </x:c>
-      <x:c r="P30" s="34" t="str"/>
+      <x:c r="P30" s="34"/>
       <x:c r="Q30" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -2670,7 +2688,7 @@
       <x:c r="O31" s="34" t="str">
         <x:v>S3-EV-009A</x:v>
       </x:c>
-      <x:c r="P31" s="34" t="str"/>
+      <x:c r="P31" s="34"/>
       <x:c r="Q31" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -2722,7 +2740,7 @@
       <x:c r="O32" s="34" t="str">
         <x:v>S3-EV-009A</x:v>
       </x:c>
-      <x:c r="P32" s="34" t="str"/>
+      <x:c r="P32" s="34"/>
       <x:c r="Q32" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -2774,7 +2792,7 @@
       <x:c r="O33" s="34" t="str">
         <x:v>S3-EV-004A</x:v>
       </x:c>
-      <x:c r="P33" s="34" t="str"/>
+      <x:c r="P33" s="34"/>
       <x:c r="Q33" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -2826,7 +2844,7 @@
       <x:c r="O34" s="34" t="str">
         <x:v>S3-EV-004A</x:v>
       </x:c>
-      <x:c r="P34" s="34" t="str"/>
+      <x:c r="P34" s="34"/>
       <x:c r="Q34" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -2878,7 +2896,7 @@
       <x:c r="O35" s="34" t="str">
         <x:v>S3-EV-004A</x:v>
       </x:c>
-      <x:c r="P35" s="34" t="str"/>
+      <x:c r="P35" s="34"/>
       <x:c r="Q35" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -2930,7 +2948,7 @@
       <x:c r="O36" s="34" t="str">
         <x:v>S3-EV-004A</x:v>
       </x:c>
-      <x:c r="P36" s="34" t="str"/>
+      <x:c r="P36" s="34"/>
       <x:c r="Q36" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -2982,7 +3000,7 @@
       <x:c r="O37" s="34" t="str">
         <x:v>S3-EV-004A</x:v>
       </x:c>
-      <x:c r="P37" s="34" t="str"/>
+      <x:c r="P37" s="34"/>
       <x:c r="Q37" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -3034,7 +3052,7 @@
       <x:c r="O38" s="34" t="str">
         <x:v>S3-EV-004A</x:v>
       </x:c>
-      <x:c r="P38" s="34" t="str"/>
+      <x:c r="P38" s="34"/>
       <x:c r="Q38" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -3086,7 +3104,7 @@
       <x:c r="O39" s="34" t="str">
         <x:v>S3-EV-004A</x:v>
       </x:c>
-      <x:c r="P39" s="34" t="str"/>
+      <x:c r="P39" s="34"/>
       <x:c r="Q39" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -3138,7 +3156,7 @@
       <x:c r="O40" s="34" t="str">
         <x:v>S3-EV-004A</x:v>
       </x:c>
-      <x:c r="P40" s="34" t="str"/>
+      <x:c r="P40" s="34"/>
       <x:c r="Q40" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -3190,7 +3208,7 @@
       <x:c r="O41" s="34" t="str">
         <x:v>S3-EV-004A</x:v>
       </x:c>
-      <x:c r="P41" s="34" t="str"/>
+      <x:c r="P41" s="34"/>
       <x:c r="Q41" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -3242,7 +3260,7 @@
       <x:c r="O42" s="34" t="str">
         <x:v>S3-EV-004A; S3-EV-009A</x:v>
       </x:c>
-      <x:c r="P42" s="34" t="str"/>
+      <x:c r="P42" s="34"/>
       <x:c r="Q42" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -3285,18 +3303,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L43" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M43" s="34" t="str">
-        <x:v>WBS 6.5 implementation/merge; WBS 6.4 for cover-letter integration where applicable</x:v>
-      </x:c>
-      <x:c r="N43" s="34" t="str"/>
-      <x:c r="O43" s="34" t="str"/>
-      <x:c r="P43" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M43" s="34"/>
+      <x:c r="N43" s="34" t="str">
+        <x:v>PASS at formal closeout. Resume Builder loaded successfully for an authenticated Student during WBS 6.5 manual UI verification and later integrated workflow verification.</x:v>
+      </x:c>
+      <x:c r="O43" s="34" t="str">
+        <x:v>S3-EV-005</x:v>
+      </x:c>
+      <x:c r="P43" s="34"/>
       <x:c r="Q43" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R43" s="34" t="str"/>
+      <x:c r="R43" s="34" t="str">
+        <x:v>Accepted from PR #59 WBS 6.5 verification and, where required, PR #78 / final WBS 7.9 successor integration evidence.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="34" t="str">
@@ -3333,18 +3355,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L44" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M44" s="34" t="str">
-        <x:v>WBS 6.5 implementation/merge; WBS 6.4 for cover-letter integration where applicable</x:v>
-      </x:c>
-      <x:c r="N44" s="34" t="str"/>
-      <x:c r="O44" s="34" t="str"/>
-      <x:c r="P44" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M44" s="34"/>
+      <x:c r="N44" s="34" t="str">
+        <x:v>PASS at formal closeout. Resume generation from the frontend to the approved backend flow was verified during WBS 6.5 and later integrated Student workflow verification.</x:v>
+      </x:c>
+      <x:c r="O44" s="34" t="str">
+        <x:v>S3-EV-005</x:v>
+      </x:c>
+      <x:c r="P44" s="34"/>
       <x:c r="Q44" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R44" s="34" t="str"/>
+      <x:c r="R44" s="34" t="str">
+        <x:v>Accepted from PR #59 WBS 6.5 verification and, where required, PR #78 / final WBS 7.9 successor integration evidence.</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="34" t="str">
@@ -3381,18 +3407,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L45" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M45" s="34" t="str">
-        <x:v>WBS 6.5 implementation/merge; WBS 6.4 for cover-letter integration where applicable</x:v>
-      </x:c>
-      <x:c r="N45" s="34" t="str"/>
-      <x:c r="O45" s="34" t="str"/>
-      <x:c r="P45" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M45" s="34"/>
+      <x:c r="N45" s="34" t="str">
+        <x:v>PASS at formal closeout. Editable Resume draft behaviour and document actions were verified during WBS 6.5 interface verification and later integrated workflow verification.</x:v>
+      </x:c>
+      <x:c r="O45" s="34" t="str">
+        <x:v>S3-EV-005</x:v>
+      </x:c>
+      <x:c r="P45" s="34"/>
       <x:c r="Q45" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R45" s="34" t="str"/>
+      <x:c r="R45" s="34" t="str">
+        <x:v>Accepted from PR #59 WBS 6.5 verification and, where required, PR #78 / final WBS 7.9 successor integration evidence.</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="34" t="str">
@@ -3429,18 +3459,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L46" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M46" s="34" t="str">
-        <x:v>WBS 6.5 implementation/merge; WBS 6.4 for cover-letter integration where applicable</x:v>
-      </x:c>
-      <x:c r="N46" s="34" t="str"/>
-      <x:c r="O46" s="34" t="str"/>
-      <x:c r="P46" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M46" s="34"/>
+      <x:c r="N46" s="34" t="str">
+        <x:v>PASS at formal closeout. Resume loading and controlled provider-error behaviour are accepted from the verified WBS 6.5 provider seam and later Sprint 4 controlled AI-error integration coverage.</x:v>
+      </x:c>
+      <x:c r="O46" s="34" t="str">
+        <x:v>S3-EV-005</x:v>
+      </x:c>
+      <x:c r="P46" s="34"/>
       <x:c r="Q46" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R46" s="34" t="str"/>
+      <x:c r="R46" s="34" t="str">
+        <x:v>Accepted from PR #59 WBS 6.5 verification and, where required, PR #78 / final WBS 7.9 successor integration evidence.</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="34" t="str">
@@ -3477,18 +3511,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L47" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M47" s="34" t="str">
-        <x:v>WBS 6.5 implementation/merge; WBS 6.4 for cover-letter integration where applicable</x:v>
-      </x:c>
-      <x:c r="N47" s="34" t="str"/>
-      <x:c r="O47" s="34" t="str"/>
-      <x:c r="P47" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M47" s="34"/>
+      <x:c r="N47" s="34" t="str">
+        <x:v>PASS at formal closeout. Cover Letter required-field behaviour, including required job information and disabled generation state, was verified in WBS 6.5.</x:v>
+      </x:c>
+      <x:c r="O47" s="34" t="str">
+        <x:v>S3-EV-005</x:v>
+      </x:c>
+      <x:c r="P47" s="34"/>
       <x:c r="Q47" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R47" s="34" t="str"/>
+      <x:c r="R47" s="34" t="str">
+        <x:v>Accepted from PR #59 WBS 6.5 verification and, where required, PR #78 / final WBS 7.9 successor integration evidence.</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="34" t="str">
@@ -3525,18 +3563,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L48" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M48" s="34" t="str">
-        <x:v>WBS 6.5 implementation/merge; WBS 6.4 for cover-letter integration where applicable</x:v>
-      </x:c>
-      <x:c r="N48" s="34" t="str"/>
-      <x:c r="O48" s="34" t="str"/>
-      <x:c r="P48" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M48" s="34"/>
+      <x:c r="N48" s="34" t="str">
+        <x:v>PASS at formal closeout. Cover Letter generation from the frontend to the approved backend flow was verified during WBS 6.5 and later integrated Student workflow verification.</x:v>
+      </x:c>
+      <x:c r="O48" s="34" t="str">
+        <x:v>S3-EV-005</x:v>
+      </x:c>
+      <x:c r="P48" s="34"/>
       <x:c r="Q48" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R48" s="34" t="str"/>
+      <x:c r="R48" s="34" t="str">
+        <x:v>Accepted from PR #59 WBS 6.5 verification and, where required, PR #78 / final WBS 7.9 successor integration evidence.</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="34" t="str">
@@ -3573,18 +3615,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L49" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M49" s="34" t="str">
-        <x:v>WBS 6.5 implementation/merge; WBS 6.4 for cover-letter integration where applicable</x:v>
-      </x:c>
-      <x:c r="N49" s="34" t="str"/>
-      <x:c r="O49" s="34" t="str"/>
-      <x:c r="P49" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M49" s="34"/>
+      <x:c r="N49" s="34" t="str">
+        <x:v>PASS at formal closeout. Editable Cover Letter draft behaviour and document actions were verified during WBS 6.5 and later integrated workflow verification.</x:v>
+      </x:c>
+      <x:c r="O49" s="34" t="str">
+        <x:v>S3-EV-005</x:v>
+      </x:c>
+      <x:c r="P49" s="34"/>
       <x:c r="Q49" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R49" s="34" t="str"/>
+      <x:c r="R49" s="34" t="str">
+        <x:v>Accepted from PR #59 WBS 6.5 verification and, where required, PR #78 / final WBS 7.9 successor integration evidence.</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="34" t="str">
@@ -3621,18 +3667,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L50" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M50" s="34" t="str">
-        <x:v>WBS 6.5 implementation/merge; WBS 6.4 for cover-letter integration where applicable</x:v>
-      </x:c>
-      <x:c r="N50" s="34" t="str"/>
-      <x:c r="O50" s="34" t="str"/>
-      <x:c r="P50" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M50" s="34"/>
+      <x:c r="N50" s="34" t="str">
+        <x:v>PASS at formal closeout. Resume and Cover Letter generated-content review and limitation states were verified in WBS 6.5 and preserved in later integration.</x:v>
+      </x:c>
+      <x:c r="O50" s="34" t="str">
+        <x:v>S3-EV-005</x:v>
+      </x:c>
+      <x:c r="P50" s="34"/>
       <x:c r="Q50" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R50" s="34" t="str"/>
+      <x:c r="R50" s="34" t="str">
+        <x:v>Accepted from PR #59 WBS 6.5 verification and, where required, PR #78 / final WBS 7.9 successor integration evidence.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="34" t="str">
@@ -3669,18 +3719,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L51" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M51" s="34" t="str">
-        <x:v>WBS 6.5 implementation/merge; WBS 6.4 for cover-letter integration where applicable</x:v>
-      </x:c>
-      <x:c r="N51" s="34" t="str"/>
-      <x:c r="O51" s="34" t="str"/>
-      <x:c r="P51" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M51" s="34"/>
+      <x:c r="N51" s="34" t="str">
+        <x:v>PASS at formal closeout. Document workflows were verified across desktop, tablet, and mobile layouts during the later integrated Student workflow verification.</x:v>
+      </x:c>
+      <x:c r="O51" s="34" t="str">
+        <x:v>S3-EV-005</x:v>
+      </x:c>
+      <x:c r="P51" s="34"/>
       <x:c r="Q51" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R51" s="34" t="str"/>
+      <x:c r="R51" s="34" t="str">
+        <x:v>Accepted from PR #59 WBS 6.5 verification and, where required, PR #78 / final WBS 7.9 successor integration evidence.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="34" t="str">
@@ -3717,18 +3771,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L52" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M52" s="34" t="str">
-        <x:v>WBS 6.5 implementation/merge; WBS 6.4 for cover-letter integration where applicable</x:v>
-      </x:c>
-      <x:c r="N52" s="34" t="str"/>
-      <x:c r="O52" s="34" t="str"/>
-      <x:c r="P52" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M52" s="34"/>
+      <x:c r="N52" s="34" t="str">
+        <x:v>PASS at formal closeout. Document form controls, HelpTip keyboard interaction, validation behaviour, and final compatibility coverage are accepted from WBS 6.5 and final Sprint 4 integration testing.</x:v>
+      </x:c>
+      <x:c r="O52" s="34" t="str">
+        <x:v>S3-EV-005</x:v>
+      </x:c>
+      <x:c r="P52" s="34"/>
       <x:c r="Q52" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R52" s="34" t="str"/>
+      <x:c r="R52" s="34" t="str">
+        <x:v>Accepted from PR #59 WBS 6.5 verification and, where required, PR #78 / final WBS 7.9 successor integration evidence.</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="34" t="str">
@@ -3767,14 +3825,14 @@
       <x:c r="L53" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M53" s="34" t="str"/>
+      <x:c r="M53" s="34"/>
       <x:c r="N53" s="34" t="str">
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O53" s="34" t="str">
         <x:v>S3-EV-002F</x:v>
       </x:c>
-      <x:c r="P53" s="34" t="str"/>
+      <x:c r="P53" s="34"/>
       <x:c r="Q53" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -3819,14 +3877,14 @@
       <x:c r="L54" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M54" s="34" t="str"/>
+      <x:c r="M54" s="34"/>
       <x:c r="N54" s="34" t="str">
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O54" s="34" t="str">
         <x:v>S3-EV-002F</x:v>
       </x:c>
-      <x:c r="P54" s="34" t="str"/>
+      <x:c r="P54" s="34"/>
       <x:c r="Q54" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -3871,14 +3929,14 @@
       <x:c r="L55" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M55" s="34" t="str"/>
+      <x:c r="M55" s="34"/>
       <x:c r="N55" s="34" t="str">
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O55" s="34" t="str">
         <x:v>S3-EV-002F</x:v>
       </x:c>
-      <x:c r="P55" s="34" t="str"/>
+      <x:c r="P55" s="34"/>
       <x:c r="Q55" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -3923,14 +3981,14 @@
       <x:c r="L56" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M56" s="34" t="str"/>
+      <x:c r="M56" s="34"/>
       <x:c r="N56" s="34" t="str">
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O56" s="34" t="str">
         <x:v>S3-EV-002F</x:v>
       </x:c>
-      <x:c r="P56" s="34" t="str"/>
+      <x:c r="P56" s="34"/>
       <x:c r="Q56" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -3975,14 +4033,14 @@
       <x:c r="L57" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M57" s="34" t="str"/>
+      <x:c r="M57" s="34"/>
       <x:c r="N57" s="34" t="str">
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O57" s="34" t="str">
         <x:v>S3-EV-002F</x:v>
       </x:c>
-      <x:c r="P57" s="34" t="str"/>
+      <x:c r="P57" s="34"/>
       <x:c r="Q57" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -4027,14 +4085,14 @@
       <x:c r="L58" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M58" s="34" t="str"/>
+      <x:c r="M58" s="34"/>
       <x:c r="N58" s="34" t="str">
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O58" s="34" t="str">
         <x:v>S3-EV-002F</x:v>
       </x:c>
-      <x:c r="P58" s="34" t="str"/>
+      <x:c r="P58" s="34"/>
       <x:c r="Q58" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -4079,14 +4137,14 @@
       <x:c r="L59" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M59" s="34" t="str"/>
+      <x:c r="M59" s="34"/>
       <x:c r="N59" s="34" t="str">
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O59" s="34" t="str">
         <x:v>S3-EV-002F</x:v>
       </x:c>
-      <x:c r="P59" s="34" t="str"/>
+      <x:c r="P59" s="34"/>
       <x:c r="Q59" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -4131,14 +4189,14 @@
       <x:c r="L60" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M60" s="34" t="str"/>
+      <x:c r="M60" s="34"/>
       <x:c r="N60" s="34" t="str">
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O60" s="34" t="str">
         <x:v>S3-EV-002F</x:v>
       </x:c>
-      <x:c r="P60" s="34" t="str"/>
+      <x:c r="P60" s="34"/>
       <x:c r="Q60" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -4183,14 +4241,14 @@
       <x:c r="L61" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M61" s="34" t="str"/>
+      <x:c r="M61" s="34"/>
       <x:c r="N61" s="34" t="str">
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O61" s="34" t="str">
         <x:v>S3-EV-002F</x:v>
       </x:c>
-      <x:c r="P61" s="34" t="str"/>
+      <x:c r="P61" s="34"/>
       <x:c r="Q61" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -4235,14 +4293,14 @@
       <x:c r="L62" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M62" s="34" t="str"/>
+      <x:c r="M62" s="34"/>
       <x:c r="N62" s="34" t="str">
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O62" s="34" t="str">
         <x:v>S3-EV-002F</x:v>
       </x:c>
-      <x:c r="P62" s="34" t="str"/>
+      <x:c r="P62" s="34"/>
       <x:c r="Q62" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -4287,14 +4345,14 @@
       <x:c r="L63" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M63" s="34" t="str"/>
+      <x:c r="M63" s="34"/>
       <x:c r="N63" s="34" t="str">
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O63" s="34" t="str">
         <x:v>S3-EV-002F</x:v>
       </x:c>
-      <x:c r="P63" s="34" t="str"/>
+      <x:c r="P63" s="34"/>
       <x:c r="Q63" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -4339,14 +4397,14 @@
       <x:c r="L64" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M64" s="34" t="str"/>
+      <x:c r="M64" s="34"/>
       <x:c r="N64" s="34" t="str">
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O64" s="34" t="str">
         <x:v>S3-EV-002F</x:v>
       </x:c>
-      <x:c r="P64" s="34" t="str"/>
+      <x:c r="P64" s="34"/>
       <x:c r="Q64" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
@@ -4391,14 +4449,14 @@
       <x:c r="L65" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M65" s="34" t="str"/>
+      <x:c r="M65" s="34"/>
       <x:c r="N65" s="34" t="str">
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O65" s="34" t="str">
         <x:v>S3-EV-002F</x:v>
       </x:c>
-      <x:c r="P65" s="34" t="str"/>
+      <x:c r="P65" s="34"/>
       <x:c r="Q65" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -4443,14 +4501,14 @@
       <x:c r="L66" s="34" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="M66" s="34" t="str"/>
+      <x:c r="M66" s="34"/>
       <x:c r="N66" s="34" t="str">
         <x:v>38/38 interview tests passed post-merge; current shared feature/sprint-3 full backend regression passed 410/410.</x:v>
       </x:c>
       <x:c r="O66" s="34" t="str">
         <x:v>S3-EV-002F; S3-EV-009A; S3-EV-009B</x:v>
       </x:c>
-      <x:c r="P66" s="34" t="str"/>
+      <x:c r="P66" s="34"/>
       <x:c r="Q66" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
@@ -4493,18 +4551,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L67" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M67" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N67" s="34" t="str"/>
-      <x:c r="O67" s="34" t="str"/>
-      <x:c r="P67" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M67" s="34"/>
+      <x:c r="N67" s="34" t="str">
+        <x:v>PASS at formal closeout. The protected Interview Preparation page was verified in the final integrated Student workflow.</x:v>
+      </x:c>
+      <x:c r="O67" s="34" t="str">
+        <x:v>S3-EV-006</x:v>
+      </x:c>
+      <x:c r="P67" s="34"/>
       <x:c r="Q67" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R67" s="34" t="str"/>
+      <x:c r="R67" s="34" t="str">
+        <x:v>PR #63 is retained as the original WBS 6.7 contribution record. Its final implementation was superseded and integrated through PR #78, with Interview AI verification also recorded in PR #74.</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="34" t="str">
@@ -4541,18 +4603,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L68" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M68" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N68" s="34" t="str"/>
-      <x:c r="O68" s="34" t="str"/>
-      <x:c r="P68" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M68" s="34"/>
+      <x:c r="N68" s="34" t="str">
+        <x:v>PASS at formal closeout. Interview question generation from the UI with target career context was verified in the final integrated workflow.</x:v>
+      </x:c>
+      <x:c r="O68" s="34" t="str">
+        <x:v>S3-EV-006</x:v>
+      </x:c>
+      <x:c r="P68" s="34"/>
       <x:c r="Q68" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R68" s="34" t="str"/>
+      <x:c r="R68" s="34" t="str">
+        <x:v>PR #63 is retained as the original WBS 6.7 contribution record. Its final implementation was superseded and integrated through PR #78, with Interview AI verification also recorded in PR #74.</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="34" t="str">
@@ -4589,18 +4655,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L69" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M69" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N69" s="34" t="str"/>
-      <x:c r="O69" s="34" t="str"/>
-      <x:c r="P69" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M69" s="34"/>
+      <x:c r="N69" s="34" t="str">
+        <x:v>PASS at formal closeout. Generated interview questions and focus areas rendered through the integrated Interview Preparation flow.</x:v>
+      </x:c>
+      <x:c r="O69" s="34" t="str">
+        <x:v>S3-EV-006</x:v>
+      </x:c>
+      <x:c r="P69" s="34"/>
       <x:c r="Q69" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R69" s="34" t="str"/>
+      <x:c r="R69" s="34" t="str">
+        <x:v>PR #63 is retained as the original WBS 6.7 contribution record. Its final implementation was superseded and integrated through PR #78, with Interview AI verification also recorded in PR #74.</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="34" t="str">
@@ -4637,18 +4707,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L70" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M70" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N70" s="34" t="str"/>
-      <x:c r="O70" s="34" t="str"/>
-      <x:c r="P70" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M70" s="34"/>
+      <x:c r="N70" s="34" t="str">
+        <x:v>PASS at formal closeout. The Student answer input retained typed answer content during the interview practice flow.</x:v>
+      </x:c>
+      <x:c r="O70" s="34" t="str">
+        <x:v>S3-EV-006</x:v>
+      </x:c>
+      <x:c r="P70" s="34"/>
       <x:c r="Q70" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R70" s="34" t="str"/>
+      <x:c r="R70" s="34" t="str">
+        <x:v>PR #63 is retained as the original WBS 6.7 contribution record. Its final implementation was superseded and integrated through PR #78, with Interview AI verification also recorded in PR #74.</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="34" t="str">
@@ -4685,18 +4759,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L71" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M71" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N71" s="34" t="str"/>
-      <x:c r="O71" s="34" t="str"/>
-      <x:c r="P71" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M71" s="34"/>
+      <x:c r="N71" s="34" t="str">
+        <x:v>PASS at formal closeout. The integrated Interview Preparation flow submitted the selected question and typed answer for feedback.</x:v>
+      </x:c>
+      <x:c r="O71" s="34" t="str">
+        <x:v>S3-EV-006</x:v>
+      </x:c>
+      <x:c r="P71" s="34"/>
       <x:c r="Q71" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R71" s="34" t="str"/>
+      <x:c r="R71" s="34" t="str">
+        <x:v>PR #63 is retained as the original WBS 6.7 contribution record. Its final implementation was superseded and integrated through PR #78, with Interview AI verification also recorded in PR #74.</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="34" t="str">
@@ -4733,18 +4811,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L72" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M72" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N72" s="34" t="str"/>
-      <x:c r="O72" s="34" t="str"/>
-      <x:c r="P72" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M72" s="34"/>
+      <x:c r="N72" s="34" t="str">
+        <x:v>PASS at formal closeout. Structured interview feedback rendered successfully in the final integrated flow.</x:v>
+      </x:c>
+      <x:c r="O72" s="34" t="str">
+        <x:v>S3-EV-006</x:v>
+      </x:c>
+      <x:c r="P72" s="34"/>
       <x:c r="Q72" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R72" s="34" t="str"/>
+      <x:c r="R72" s="34" t="str">
+        <x:v>PR #63 is retained as the original WBS 6.7 contribution record. Its final implementation was superseded and integrated through PR #78, with Interview AI verification also recorded in PR #74.</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="34" t="str">
@@ -4781,18 +4863,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L73" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M73" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N73" s="34" t="str"/>
-      <x:c r="O73" s="34" t="str"/>
-      <x:c r="P73" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M73" s="34"/>
+      <x:c r="N73" s="34" t="str">
+        <x:v>PASS at formal closeout. Interview AI review and limitation messaging was preserved in the integrated flow.</x:v>
+      </x:c>
+      <x:c r="O73" s="34" t="str">
+        <x:v>S3-EV-006</x:v>
+      </x:c>
+      <x:c r="P73" s="34"/>
       <x:c r="Q73" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R73" s="34" t="str"/>
+      <x:c r="R73" s="34" t="str">
+        <x:v>PR #63 is retained as the original WBS 6.7 contribution record. Its final implementation was superseded and integrated through PR #78, with Interview AI verification also recorded in PR #74.</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="34" t="str">
@@ -4829,18 +4915,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L74" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M74" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N74" s="34" t="str"/>
-      <x:c r="O74" s="34" t="str"/>
-      <x:c r="P74" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M74" s="34"/>
+      <x:c r="N74" s="34" t="str">
+        <x:v>PASS at formal closeout. Interview loading, validation, controlled provider-error, retry, and feedback states were verified across the later integrated implementation and Interview AI remediation.</x:v>
+      </x:c>
+      <x:c r="O74" s="34" t="str">
+        <x:v>S3-EV-006</x:v>
+      </x:c>
+      <x:c r="P74" s="34"/>
       <x:c r="Q74" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R74" s="34" t="str"/>
+      <x:c r="R74" s="34" t="str">
+        <x:v>PR #63 is retained as the original WBS 6.7 contribution record. Its final implementation was superseded and integrated through PR #78, with Interview AI verification also recorded in PR #74.</x:v>
+      </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="34" t="str">
@@ -4877,18 +4967,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L75" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M75" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N75" s="34" t="str"/>
-      <x:c r="O75" s="34" t="str"/>
-      <x:c r="P75" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M75" s="34"/>
+      <x:c r="N75" s="34" t="str">
+        <x:v>PASS at formal closeout. Interview Preparation was verified across desktop, tablet, and mobile layouts in the later integrated workflow.</x:v>
+      </x:c>
+      <x:c r="O75" s="34" t="str">
+        <x:v>S3-EV-006</x:v>
+      </x:c>
+      <x:c r="P75" s="34"/>
       <x:c r="Q75" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R75" s="34" t="str"/>
+      <x:c r="R75" s="34" t="str">
+        <x:v>PR #63 is retained as the original WBS 6.7 contribution record. Its final implementation was superseded and integrated through PR #78, with Interview AI verification also recorded in PR #74.</x:v>
+      </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="34" t="str">
@@ -4925,18 +5019,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L76" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M76" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N76" s="34" t="str"/>
-      <x:c r="O76" s="34" t="str"/>
-      <x:c r="P76" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M76" s="34"/>
+      <x:c r="N76" s="34" t="str">
+        <x:v>PASS at formal closeout. Interview keyboard and current-browser compatibility are accepted from the final Sprint 4 WBS 7.9 compatibility closeout.</x:v>
+      </x:c>
+      <x:c r="O76" s="34" t="str">
+        <x:v>S3-EV-006</x:v>
+      </x:c>
+      <x:c r="P76" s="34"/>
       <x:c r="Q76" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R76" s="34" t="str"/>
+      <x:c r="R76" s="34" t="str">
+        <x:v>PR #63 is retained as the original WBS 6.7 contribution record. Its final implementation was superseded and integrated through PR #78, with Interview AI verification also recorded in PR #74.</x:v>
+      </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="34" t="str">
@@ -4973,18 +5071,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L77" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M77" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7</x:v>
-      </x:c>
-      <x:c r="N77" s="34" t="str"/>
-      <x:c r="O77" s="34" t="str"/>
-      <x:c r="P77" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M77" s="34"/>
+      <x:c r="N77" s="34" t="str">
+        <x:v>PASS at formal closeout. WBS 6.3, 6.4, 6.5, and 6.6 were present in the Sprint 3 history. The final WBS 6.7 implementation was later superseded and integrated through PR #78 on feature/sprint-4. Formal Sprint 3 closeout accepts that verified successor integration evidence.</x:v>
+      </x:c>
+      <x:c r="O77" s="34" t="str">
+        <x:v>S3-EV-007</x:v>
+      </x:c>
+      <x:c r="P77" s="34"/>
       <x:c r="Q77" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R77" s="34" t="str"/>
+      <x:c r="R77" s="34" t="str">
+        <x:v>Formal Sprint 3 closeout uses verified successor-baseline integration evidence from PR #78 and final WBS 7.9 where the original Sprint 3 integration gate was completed later.</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="34" t="str">
@@ -5021,18 +5123,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L78" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M78" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7</x:v>
-      </x:c>
-      <x:c r="N78" s="34" t="str"/>
-      <x:c r="O78" s="34" t="str"/>
-      <x:c r="P78" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M78" s="34"/>
+      <x:c r="N78" s="34" t="str">
+        <x:v>PASS at formal closeout. Resume UI to API generation and review flow was verified in the later integrated Student workflow and final Sprint 4 end-to-end smoke.</x:v>
+      </x:c>
+      <x:c r="O78" s="34" t="str">
+        <x:v>S3-EV-007</x:v>
+      </x:c>
+      <x:c r="P78" s="34"/>
       <x:c r="Q78" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R78" s="34" t="str"/>
+      <x:c r="R78" s="34" t="str">
+        <x:v>Formal Sprint 3 closeout uses verified successor-baseline integration evidence from PR #78 and final WBS 7.9 where the original Sprint 3 integration gate was completed later.</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="34" t="str">
@@ -5069,18 +5175,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L79" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M79" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7</x:v>
-      </x:c>
-      <x:c r="N79" s="34" t="str"/>
-      <x:c r="O79" s="34" t="str"/>
-      <x:c r="P79" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M79" s="34"/>
+      <x:c r="N79" s="34" t="str">
+        <x:v>PASS at formal closeout. Cover Letter UI to API generation and review flow was verified in the later integrated Student workflow and final Sprint 4 end-to-end smoke.</x:v>
+      </x:c>
+      <x:c r="O79" s="34" t="str">
+        <x:v>S3-EV-007</x:v>
+      </x:c>
+      <x:c r="P79" s="34"/>
       <x:c r="Q79" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R79" s="34" t="str"/>
+      <x:c r="R79" s="34" t="str">
+        <x:v>Formal Sprint 3 closeout uses verified successor-baseline integration evidence from PR #78 and final WBS 7.9 where the original Sprint 3 integration gate was completed later.</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="34" t="str">
@@ -5117,18 +5227,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L80" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M80" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7</x:v>
-      </x:c>
-      <x:c r="N80" s="34" t="str"/>
-      <x:c r="O80" s="34" t="str"/>
-      <x:c r="P80" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M80" s="34"/>
+      <x:c r="N80" s="34" t="str">
+        <x:v>PASS at formal closeout. Interview question UI to API flow was verified in PR #78 and final Sprint 4 Interview regression.</x:v>
+      </x:c>
+      <x:c r="O80" s="34" t="str">
+        <x:v>S3-EV-007</x:v>
+      </x:c>
+      <x:c r="P80" s="34"/>
       <x:c r="Q80" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R80" s="34" t="str"/>
+      <x:c r="R80" s="34" t="str">
+        <x:v>Formal Sprint 3 closeout uses verified successor-baseline integration evidence from PR #78 and final WBS 7.9 where the original Sprint 3 integration gate was completed later.</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="34" t="str">
@@ -5165,18 +5279,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L81" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M81" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7</x:v>
-      </x:c>
-      <x:c r="N81" s="34" t="str"/>
-      <x:c r="O81" s="34" t="str"/>
-      <x:c r="P81" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M81" s="34"/>
+      <x:c r="N81" s="34" t="str">
+        <x:v>PASS at formal closeout. Interview feedback UI to API flow was verified in PR #78, PR #74, and final Sprint 4 Interview regression.</x:v>
+      </x:c>
+      <x:c r="O81" s="34" t="str">
+        <x:v>S3-EV-007</x:v>
+      </x:c>
+      <x:c r="P81" s="34"/>
       <x:c r="Q81" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R81" s="34" t="str"/>
+      <x:c r="R81" s="34" t="str">
+        <x:v>Formal Sprint 3 closeout uses verified successor-baseline integration evidence from PR #78 and final WBS 7.9 where the original Sprint 3 integration gate was completed later.</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="34" t="str">
@@ -5213,18 +5331,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L82" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M82" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7</x:v>
-      </x:c>
-      <x:c r="N82" s="34" t="str"/>
-      <x:c r="O82" s="34" t="str"/>
-      <x:c r="P82" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M82" s="34"/>
+      <x:c r="N82" s="34" t="str">
+        <x:v>PASS at formal closeout. Student-context privacy and ownership controls are accepted from the integrated Student workflow privacy verification and final Sprint 4 security/privacy regression coverage.</x:v>
+      </x:c>
+      <x:c r="O82" s="34" t="str">
+        <x:v>S3-EV-007</x:v>
+      </x:c>
+      <x:c r="P82" s="34"/>
       <x:c r="Q82" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R82" s="34" t="str"/>
+      <x:c r="R82" s="34" t="str">
+        <x:v>Formal Sprint 3 closeout uses verified successor-baseline integration evidence from PR #78 and final WBS 7.9 where the original Sprint 3 integration gate was completed later.</x:v>
+      </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="34" t="str">
@@ -5261,18 +5383,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L83" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M83" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7</x:v>
-      </x:c>
-      <x:c r="N83" s="34" t="str"/>
-      <x:c r="O83" s="34" t="str"/>
-      <x:c r="P83" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M83" s="34"/>
+      <x:c r="N83" s="34" t="str">
+        <x:v>PASS at formal closeout. Resume ownership and prompt-manipulation protections are accepted from Sprint 3 backend safety tests plus final successor security and integration verification.</x:v>
+      </x:c>
+      <x:c r="O83" s="34" t="str">
+        <x:v>S3-EV-007</x:v>
+      </x:c>
+      <x:c r="P83" s="34"/>
       <x:c r="Q83" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R83" s="34" t="str"/>
+      <x:c r="R83" s="34" t="str">
+        <x:v>Formal Sprint 3 closeout uses verified successor-baseline integration evidence from PR #78 and final WBS 7.9 where the original Sprint 3 integration gate was completed later.</x:v>
+      </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="34" t="str">
@@ -5309,18 +5435,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L84" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M84" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7</x:v>
-      </x:c>
-      <x:c r="N84" s="34" t="str"/>
-      <x:c r="O84" s="34" t="str"/>
-      <x:c r="P84" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M84" s="34"/>
+      <x:c r="N84" s="34" t="str">
+        <x:v>PASS at formal closeout. Cover Letter job-description trust boundaries and prompt-injection protections are accepted from Sprint 3 safety tests plus later integrated validation.</x:v>
+      </x:c>
+      <x:c r="O84" s="34" t="str">
+        <x:v>S3-EV-007</x:v>
+      </x:c>
+      <x:c r="P84" s="34"/>
       <x:c r="Q84" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R84" s="34" t="str"/>
+      <x:c r="R84" s="34" t="str">
+        <x:v>Formal Sprint 3 closeout uses verified successor-baseline integration evidence from PR #78 and final WBS 7.9 where the original Sprint 3 integration gate was completed later.</x:v>
+      </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="34" t="str">
@@ -5357,18 +5487,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L85" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M85" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7</x:v>
-      </x:c>
-      <x:c r="N85" s="34" t="str"/>
-      <x:c r="O85" s="34" t="str"/>
-      <x:c r="P85" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M85" s="34"/>
+      <x:c r="N85" s="34" t="str">
+        <x:v>PASS at formal closeout. Interview untrusted-input and safety-contract behaviour is accepted from Sprint 3 API safety tests and later Interview AI validation.</x:v>
+      </x:c>
+      <x:c r="O85" s="34" t="str">
+        <x:v>S3-EV-007</x:v>
+      </x:c>
+      <x:c r="P85" s="34"/>
       <x:c r="Q85" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R85" s="34" t="str"/>
+      <x:c r="R85" s="34" t="str">
+        <x:v>Formal Sprint 3 closeout uses verified successor-baseline integration evidence from PR #78 and final WBS 7.9 where the original Sprint 3 integration gate was completed later.</x:v>
+      </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="34" t="str">
@@ -5405,18 +5539,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L86" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M86" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7</x:v>
-      </x:c>
-      <x:c r="N86" s="34" t="str"/>
-      <x:c r="O86" s="34" t="str"/>
-      <x:c r="P86" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M86" s="34"/>
+      <x:c r="N86" s="34" t="str">
+        <x:v>PASS at formal closeout. Review-required and AI limitation states are accepted from the verified Resume, Cover Letter, and Interview integrated workflows.</x:v>
+      </x:c>
+      <x:c r="O86" s="34" t="str">
+        <x:v>S3-EV-007</x:v>
+      </x:c>
+      <x:c r="P86" s="34"/>
       <x:c r="Q86" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R86" s="34" t="str"/>
+      <x:c r="R86" s="34" t="str">
+        <x:v>Formal Sprint 3 closeout uses verified successor-baseline integration evidence from PR #78 and final WBS 7.9 where the original Sprint 3 integration gate was completed later.</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="34" t="str">
@@ -5453,18 +5591,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L87" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M87" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7</x:v>
-      </x:c>
-      <x:c r="N87" s="34" t="str"/>
-      <x:c r="O87" s="34" t="str"/>
-      <x:c r="P87" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M87" s="34"/>
+      <x:c r="N87" s="34" t="str">
+        <x:v>PASS at formal closeout. Controlled provider-unavailable and validation-error handling was verified across the document and Interview service boundaries and later Sprint 4 AI integration.</x:v>
+      </x:c>
+      <x:c r="O87" s="34" t="str">
+        <x:v>S3-EV-007</x:v>
+      </x:c>
+      <x:c r="P87" s="34"/>
       <x:c r="Q87" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R87" s="34" t="str"/>
+      <x:c r="R87" s="34" t="str">
+        <x:v>Formal Sprint 3 closeout uses verified successor-baseline integration evidence from PR #78 and final WBS 7.9 where the original Sprint 3 integration gate was completed later.</x:v>
+      </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="34" t="str">
@@ -5501,18 +5643,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L88" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M88" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7</x:v>
-      </x:c>
-      <x:c r="N88" s="34" t="str"/>
-      <x:c r="O88" s="34" t="str"/>
-      <x:c r="P88" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M88" s="34"/>
+      <x:c r="N88" s="34" t="str">
+        <x:v>PASS at formal closeout. Protected document and Interview flows and invalid-authentication handling are accepted from Sprint 3 API checks and final authentication/security regression.</x:v>
+      </x:c>
+      <x:c r="O88" s="34" t="str">
+        <x:v>S3-EV-007</x:v>
+      </x:c>
+      <x:c r="P88" s="34"/>
       <x:c r="Q88" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R88" s="34" t="str"/>
+      <x:c r="R88" s="34" t="str">
+        <x:v>Formal Sprint 3 closeout uses verified successor-baseline integration evidence from PR #78 and final WBS 7.9 where the original Sprint 3 integration gate was completed later.</x:v>
+      </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="34" t="str">
@@ -5549,18 +5695,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L89" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M89" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7</x:v>
-      </x:c>
-      <x:c r="N89" s="34" t="str"/>
-      <x:c r="O89" s="34" t="str"/>
-      <x:c r="P89" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M89" s="34"/>
+      <x:c r="N89" s="34" t="str">
+        <x:v>PASS at formal closeout. Student navigation and context handling across Resume, Cover Letter, Job Matching, and Interview Preparation were verified in the later integrated Student workflow.</x:v>
+      </x:c>
+      <x:c r="O89" s="34" t="str">
+        <x:v>S3-EV-007</x:v>
+      </x:c>
+      <x:c r="P89" s="34"/>
       <x:c r="Q89" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R89" s="34" t="str"/>
+      <x:c r="R89" s="34" t="str">
+        <x:v>Formal Sprint 3 closeout uses verified successor-baseline integration evidence from PR #78 and final WBS 7.9 where the original Sprint 3 integration gate was completed later.</x:v>
+      </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="34" t="str">
@@ -5597,18 +5747,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L90" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M90" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7</x:v>
-      </x:c>
-      <x:c r="N90" s="34" t="str"/>
-      <x:c r="O90" s="34" t="str"/>
-      <x:c r="P90" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M90" s="34"/>
+      <x:c r="N90" s="34" t="str">
+        <x:v>PASS at formal closeout. The core Student journey covering authentication, Resume, Cover Letter, and Interview functions was verified through PR #78 and the final Sprint 4 feature-complete smoke.</x:v>
+      </x:c>
+      <x:c r="O90" s="34" t="str">
+        <x:v>S3-EV-007</x:v>
+      </x:c>
+      <x:c r="P90" s="34"/>
       <x:c r="Q90" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R90" s="34" t="str"/>
+      <x:c r="R90" s="34" t="str">
+        <x:v>Formal Sprint 3 closeout uses verified successor-baseline integration evidence from PR #78 and final WBS 7.9 where the original Sprint 3 integration gate was completed later.</x:v>
+      </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="34" t="str">
@@ -5645,23 +5799,21 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L91" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M91" s="34" t="str">
-        <x:v>WBS 6.8</x:v>
-      </x:c>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M91" s="34"/>
       <x:c r="N91" s="34" t="str">
-        <x:v>Interim pre-WBS 6.8 shared backend baseline passed 410/410 tests on feature/sprint-3.</x:v>
+        <x:v>PASS at formal closeout. PR #78 reports a full backend regression of 1058 tests passed.</x:v>
       </x:c>
       <x:c r="O91" s="34" t="str">
-        <x:v>S3-EV-009A</x:v>
-      </x:c>
-      <x:c r="P91" s="34" t="str"/>
+        <x:v>S3-EV-008</x:v>
+      </x:c>
+      <x:c r="P91" s="34"/>
       <x:c r="Q91" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R91" s="34" t="str">
-        <x:v>Status remains Blocked because the final WBS 6.9 regression must run after WBS 6.8 integration.</x:v>
+        <x:v>Formal closeout regression and evidence reconciliation. Later verified successor evidence is used where final Sprint 3 integration occurred during Sprint 4.</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -5699,23 +5851,21 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L92" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M92" s="34" t="str">
-        <x:v>WBS 6.8</x:v>
-      </x:c>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M92" s="34"/>
       <x:c r="N92" s="34" t="str">
-        <x:v>Interim Django system check passed with no issues on feature/sprint-3.</x:v>
+        <x:v>PASS at formal closeout. PR #74 records Django system check PASS on the later integrated baseline.</x:v>
       </x:c>
       <x:c r="O92" s="34" t="str">
-        <x:v>S3-EV-009B</x:v>
-      </x:c>
-      <x:c r="P92" s="34" t="str"/>
+        <x:v>S3-EV-008</x:v>
+      </x:c>
+      <x:c r="P92" s="34"/>
       <x:c r="Q92" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R92" s="34" t="str">
-        <x:v>Status remains Blocked because this check must be rerun after WBS 6.8 integration.</x:v>
+        <x:v>Formal closeout regression and evidence reconciliation. Later verified successor evidence is used where final Sprint 3 integration occurred during Sprint 4.</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -5753,23 +5903,21 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L93" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M93" s="34" t="str">
-        <x:v>WBS 6.8</x:v>
-      </x:c>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M93" s="34"/>
       <x:c r="N93" s="34" t="str">
-        <x:v>Interim makemigrations --check reported no changes on feature/sprint-3.</x:v>
+        <x:v>PASS at formal closeout. PR #74 records migration state PASS and migration drift with no changes detected.</x:v>
       </x:c>
       <x:c r="O93" s="34" t="str">
-        <x:v>S3-EV-009B</x:v>
-      </x:c>
-      <x:c r="P93" s="34" t="str"/>
+        <x:v>S3-EV-008</x:v>
+      </x:c>
+      <x:c r="P93" s="34"/>
       <x:c r="Q93" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
       <x:c r="R93" s="34" t="str">
-        <x:v>Status remains Blocked because final migration verification belongs to post-WBS 6.8 Sprint 3 testing.</x:v>
+        <x:v>Formal closeout regression and evidence reconciliation. Later verified successor evidence is used where final Sprint 3 integration occurred during Sprint 4.</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -5807,18 +5955,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L94" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M94" s="34" t="str">
-        <x:v>WBS 6.8</x:v>
-      </x:c>
-      <x:c r="N94" s="34" t="str"/>
-      <x:c r="O94" s="34" t="str"/>
-      <x:c r="P94" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M94" s="34"/>
+      <x:c r="N94" s="34" t="str">
+        <x:v>PASS at formal closeout. PR #78 records frontend lint with 0 warnings and 0 errors.</x:v>
+      </x:c>
+      <x:c r="O94" s="34" t="str">
+        <x:v>S3-EV-008</x:v>
+      </x:c>
+      <x:c r="P94" s="34"/>
       <x:c r="Q94" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R94" s="34" t="str"/>
+      <x:c r="R94" s="34" t="str">
+        <x:v>Formal closeout regression and evidence reconciliation. Later verified successor evidence is used where final Sprint 3 integration occurred during Sprint 4.</x:v>
+      </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="34" t="str">
@@ -5855,18 +6007,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L95" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M95" s="34" t="str">
-        <x:v>WBS 6.8</x:v>
-      </x:c>
-      <x:c r="N95" s="34" t="str"/>
-      <x:c r="O95" s="34" t="str"/>
-      <x:c r="P95" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M95" s="34"/>
+      <x:c r="N95" s="34" t="str">
+        <x:v>PASS at formal closeout. PR #78 records a successful frontend production build.</x:v>
+      </x:c>
+      <x:c r="O95" s="34" t="str">
+        <x:v>S3-EV-008</x:v>
+      </x:c>
+      <x:c r="P95" s="34"/>
       <x:c r="Q95" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R95" s="34" t="str"/>
+      <x:c r="R95" s="34" t="str">
+        <x:v>Formal closeout regression and evidence reconciliation. Later verified successor evidence is used where final Sprint 3 integration occurred during Sprint 4.</x:v>
+      </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="34" t="str">
@@ -5903,18 +6059,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L96" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M96" s="34" t="str">
-        <x:v>WBS 6.8</x:v>
-      </x:c>
-      <x:c r="N96" s="34" t="str"/>
-      <x:c r="O96" s="34" t="str"/>
-      <x:c r="P96" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M96" s="34"/>
+      <x:c r="N96" s="34" t="str">
+        <x:v>PASS at formal closeout. Final Sprint 4 S4-REG-01 authentication regression passed.</x:v>
+      </x:c>
+      <x:c r="O96" s="34" t="str">
+        <x:v>S3-EV-008</x:v>
+      </x:c>
+      <x:c r="P96" s="34"/>
       <x:c r="Q96" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R96" s="34" t="str"/>
+      <x:c r="R96" s="34" t="str">
+        <x:v>Formal closeout regression and evidence reconciliation. Later verified successor evidence is used where final Sprint 3 integration occurred during Sprint 4.</x:v>
+      </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="34" t="str">
@@ -5951,18 +6111,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L97" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M97" s="34" t="str">
-        <x:v>WBS 6.8</x:v>
-      </x:c>
-      <x:c r="N97" s="34" t="str"/>
-      <x:c r="O97" s="34" t="str"/>
-      <x:c r="P97" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M97" s="34"/>
+      <x:c r="N97" s="34" t="str">
+        <x:v>PASS at formal closeout. Student Profile regression, persistence, and privacy were included in later integrated manual regression and final WBS 7.9 verification.</x:v>
+      </x:c>
+      <x:c r="O97" s="34" t="str">
+        <x:v>S3-EV-008</x:v>
+      </x:c>
+      <x:c r="P97" s="34"/>
       <x:c r="Q97" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R97" s="34" t="str"/>
+      <x:c r="R97" s="34" t="str">
+        <x:v>Formal closeout regression and evidence reconciliation. Later verified successor evidence is used where final Sprint 3 integration occurred during Sprint 4.</x:v>
+      </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="34" t="str">
@@ -5999,18 +6163,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L98" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M98" s="34" t="str">
-        <x:v>WBS 6.8</x:v>
-      </x:c>
-      <x:c r="N98" s="34" t="str"/>
-      <x:c r="O98" s="34" t="str"/>
-      <x:c r="P98" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M98" s="34"/>
+      <x:c r="N98" s="34" t="str">
+        <x:v>PASS at formal closeout. Final Sprint 4 S4-REG-03 career-analysis regression passed.</x:v>
+      </x:c>
+      <x:c r="O98" s="34" t="str">
+        <x:v>S3-EV-008</x:v>
+      </x:c>
+      <x:c r="P98" s="34"/>
       <x:c r="Q98" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R98" s="34" t="str"/>
+      <x:c r="R98" s="34" t="str">
+        <x:v>Formal closeout regression and evidence reconciliation. Later verified successor evidence is used where final Sprint 3 integration occurred during Sprint 4.</x:v>
+      </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="34" t="str">
@@ -6047,18 +6215,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L99" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M99" s="34" t="str">
-        <x:v>WBS 6.8</x:v>
-      </x:c>
-      <x:c r="N99" s="34" t="str"/>
-      <x:c r="O99" s="34" t="str"/>
-      <x:c r="P99" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M99" s="34"/>
+      <x:c r="N99" s="34" t="str">
+        <x:v>PASS at formal closeout. Chrome compatibility is accepted from final Sprint 4 WBS 7.9 compatibility testing, where all 129 planned Sprint 4 cases passed.</x:v>
+      </x:c>
+      <x:c r="O99" s="34" t="str">
+        <x:v>S3-EV-008</x:v>
+      </x:c>
+      <x:c r="P99" s="34"/>
       <x:c r="Q99" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R99" s="34" t="str"/>
+      <x:c r="R99" s="34" t="str">
+        <x:v>Formal closeout regression and evidence reconciliation. Later verified successor evidence is used where final Sprint 3 integration occurred during Sprint 4.</x:v>
+      </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="34" t="str">
@@ -6095,18 +6267,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L100" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M100" s="34" t="str">
-        <x:v>WBS 6.8</x:v>
-      </x:c>
-      <x:c r="N100" s="34" t="str"/>
-      <x:c r="O100" s="34" t="str"/>
-      <x:c r="P100" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M100" s="34"/>
+      <x:c r="N100" s="34" t="str">
+        <x:v>PASS at formal closeout. Edge compatibility is accepted from final Sprint 4 WBS 7.9 compatibility testing, where all 129 planned Sprint 4 cases passed.</x:v>
+      </x:c>
+      <x:c r="O100" s="34" t="str">
+        <x:v>S3-EV-008</x:v>
+      </x:c>
+      <x:c r="P100" s="34"/>
       <x:c r="Q100" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R100" s="34" t="str"/>
+      <x:c r="R100" s="34" t="str">
+        <x:v>Formal closeout regression and evidence reconciliation. Later verified successor evidence is used where final Sprint 3 integration occurred during Sprint 4.</x:v>
+      </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="34" t="str">
@@ -6143,18 +6319,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L101" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M101" s="34" t="str">
-        <x:v>WBS 6.8</x:v>
-      </x:c>
-      <x:c r="N101" s="34" t="str"/>
-      <x:c r="O101" s="34" t="str"/>
-      <x:c r="P101" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M101" s="34"/>
+      <x:c r="N101" s="34" t="str">
+        <x:v>PASS at formal closeout. Firefox compatibility is accepted from final Sprint 4 WBS 7.9 compatibility testing, where all 129 planned Sprint 4 cases passed.</x:v>
+      </x:c>
+      <x:c r="O101" s="34" t="str">
+        <x:v>S3-EV-008</x:v>
+      </x:c>
+      <x:c r="P101" s="34"/>
       <x:c r="Q101" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R101" s="34" t="str"/>
+      <x:c r="R101" s="34" t="str">
+        <x:v>Formal closeout regression and evidence reconciliation. Later verified successor evidence is used where final Sprint 3 integration occurred during Sprint 4.</x:v>
+      </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="34" t="str">
@@ -6191,18 +6371,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L102" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M102" s="34" t="str">
-        <x:v>WBS 6.8</x:v>
-      </x:c>
-      <x:c r="N102" s="34" t="str"/>
-      <x:c r="O102" s="34" t="str"/>
-      <x:c r="P102" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M102" s="34"/>
+      <x:c r="N102" s="34" t="str">
+        <x:v>PASS at formal closeout. PR #78 records manual verification at desktop, tablet, and mobile layouts, with final WBS 7.9 responsive checks completed.</x:v>
+      </x:c>
+      <x:c r="O102" s="34" t="str">
+        <x:v>S3-EV-008</x:v>
+      </x:c>
+      <x:c r="P102" s="34"/>
       <x:c r="Q102" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R102" s="34" t="str"/>
+      <x:c r="R102" s="34" t="str">
+        <x:v>Formal closeout regression and evidence reconciliation. Later verified successor evidence is used where final Sprint 3 integration occurred during Sprint 4.</x:v>
+      </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="34" t="str">
@@ -6239,18 +6423,22 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L103" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M103" s="34" t="str">
-        <x:v>WBS 6.8</x:v>
-      </x:c>
-      <x:c r="N103" s="34" t="str"/>
-      <x:c r="O103" s="34" t="str"/>
-      <x:c r="P103" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M103" s="34"/>
+      <x:c r="N103" s="34" t="str">
+        <x:v>PASS at formal closeout. Accessibility basics are accepted from the final WBS 7.9 closeout, which completed all planned Sprint 4 test cases as Pass.</x:v>
+      </x:c>
+      <x:c r="O103" s="34" t="str">
+        <x:v>S3-EV-008</x:v>
+      </x:c>
+      <x:c r="P103" s="34"/>
       <x:c r="Q103" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R103" s="34" t="str"/>
+      <x:c r="R103" s="34" t="str">
+        <x:v>Formal closeout regression and evidence reconciliation. Later verified successor evidence is used where final Sprint 3 integration occurred during Sprint 4.</x:v>
+      </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="34" t="str">
@@ -6287,18 +6475,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L104" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M104" s="34" t="str">
-        <x:v>WBS 6.8</x:v>
-      </x:c>
-      <x:c r="N104" s="34" t="str"/>
-      <x:c r="O104" s="34" t="str"/>
-      <x:c r="P104" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M104" s="34"/>
+      <x:c r="N104" s="34" t="str">
+        <x:v>PASS at formal closeout. PR #74 verified controlled provider failure and timeout handling, PR #78 verified user-facing AI workflow states, and final WBS 7.9 provider-failure coverage passed.</x:v>
+      </x:c>
+      <x:c r="O104" s="34" t="str">
+        <x:v>S3-EV-008</x:v>
+      </x:c>
+      <x:c r="P104" s="34"/>
       <x:c r="Q104" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R104" s="34" t="str"/>
+      <x:c r="R104" s="34" t="str">
+        <x:v>Formal closeout regression and evidence reconciliation. Later verified successor evidence is used where final Sprint 3 integration occurred during Sprint 4.</x:v>
+      </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="34" t="str">
@@ -6335,18 +6527,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L105" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M105" s="34" t="str">
-        <x:v>WBS 6.8</x:v>
-      </x:c>
-      <x:c r="N105" s="34" t="str"/>
-      <x:c r="O105" s="34" t="str"/>
-      <x:c r="P105" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M105" s="34"/>
+      <x:c r="N105" s="34" t="str">
+        <x:v>PASS. Formal Sprint 3 closeout reconciled all 100 test cases, updated S3-EV-005 through S3-EV-008, recorded successor verification references, and left no Fail, Blocked, Not Run, or Retest cases.</x:v>
+      </x:c>
+      <x:c r="O105" s="34" t="str">
+        <x:v>S3-EV-008</x:v>
+      </x:c>
+      <x:c r="P105" s="34"/>
       <x:c r="Q105" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R105" s="34" t="str"/>
+      <x:c r="R105" s="34" t="str">
+        <x:v>Formal closeout regression and evidence reconciliation. Later verified successor evidence is used where final Sprint 3 integration occurred during Sprint 4.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6387,7 +6583,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74920cca6980474d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc98bcfffad094cf9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6832,124 +7028,132 @@
         <x:v>Fresh post-merge evidence: 48/48 documents tests passed in 31.948s; exit code 0.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="54" customHeight="1">
       <x:c r="A18" s="34" t="str">
         <x:v>S3-EV-005</x:v>
       </x:c>
       <x:c r="B18" s="34" t="str">
-        <x:v>TBD</x:v>
+        <x:v>S3-TC-004:S3-TC-005; S3-TC-038:S3-TC-047</x:v>
       </x:c>
       <x:c r="C18" s="34" t="str">
-        <x:v>6.5</x:v>
+        <x:v>6.5/6.9</x:v>
       </x:c>
       <x:c r="D18" s="34" t="str">
-        <x:v>Screenshot</x:v>
+        <x:v>Closeout traceability</x:v>
       </x:c>
       <x:c r="E18" s="34" t="str">
-        <x:v>Resume and cover-letter interface evidence</x:v>
+        <x:v>Document interface, frontend lint/build, responsive and accessibility verification accepted from verified implementation and later integrated workflow evidence</x:v>
       </x:c>
       <x:c r="F18" s="34" t="str">
-        <x:v>docs/testing/evidence/sprint-3/S3-EV-005-*</x:v>
+        <x:v>PR #59: https://github.com/JeraldBucud/GradNavi/pull/59 | PR #78: https://github.com/JeraldBucud/GradNavi/pull/78</x:v>
       </x:c>
       <x:c r="G18" s="34" t="str">
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="H18" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="I18" s="79" t="str"/>
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I18" s="84" t="n">
+        <x:v>46304</x:v>
+      </x:c>
       <x:c r="J18" s="34" t="str">
-        <x:v>Blocked until WBS 6.5 ready</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
+        <x:v>Formal Sprint 3 closeout accepts verified later integration evidence. No rerun was requested during closeout.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="54" customHeight="1">
       <x:c r="A19" s="34" t="str">
         <x:v>S3-EV-006</x:v>
       </x:c>
       <x:c r="B19" s="34" t="str">
-        <x:v>TBD</x:v>
+        <x:v>S3-TC-062:S3-TC-071</x:v>
       </x:c>
       <x:c r="C19" s="34" t="str">
         <x:v>6.7</x:v>
       </x:c>
       <x:c r="D19" s="34" t="str">
-        <x:v>Screenshot</x:v>
+        <x:v>Closeout traceability</x:v>
       </x:c>
       <x:c r="E19" s="34" t="str">
-        <x:v>Interview preparation interface evidence</x:v>
+        <x:v>Interview Preparation interface, question/answer flow, feedback, error handling, responsive behaviour and compatibility accepted from later integrated implementation</x:v>
       </x:c>
       <x:c r="F19" s="34" t="str">
-        <x:v>docs/testing/evidence/sprint-3/S3-EV-006-*</x:v>
+        <x:v>PR #63: https://github.com/JeraldBucud/GradNavi/pull/63 | PR #74: https://github.com/JeraldBucud/GradNavi/pull/74 | PR #78: https://github.com/JeraldBucud/GradNavi/pull/78</x:v>
       </x:c>
       <x:c r="G19" s="34" t="str">
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="H19" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="I19" s="79" t="str"/>
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I19" s="84" t="n">
+        <x:v>46304</x:v>
+      </x:c>
       <x:c r="J19" s="34" t="str">
-        <x:v>Blocked until WBS 6.7 ready</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
+        <x:v>PR #63 closed without merge to feature/sprint-3. The final WBS 6.7 implementation was superseded and integrated through PR #78; PR #74 records later Interview AI validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="54" customHeight="1">
       <x:c r="A20" s="34" t="str">
         <x:v>S3-EV-007</x:v>
       </x:c>
       <x:c r="B20" s="34" t="str">
-        <x:v>TBD</x:v>
+        <x:v>S3-TC-001; S3-TC-072:S3-TC-085</x:v>
       </x:c>
       <x:c r="C20" s="34" t="str">
         <x:v>6.8</x:v>
       </x:c>
       <x:c r="D20" s="34" t="str">
-        <x:v>Integration</x:v>
+        <x:v>Integration closeout</x:v>
       </x:c>
       <x:c r="E20" s="34" t="str">
-        <x:v>Sprint 3 end-to-end integration evidence</x:v>
+        <x:v>Sprint 3 end-to-end integration, Student context, security, review-state and core-flow verification accepted from the verified successor integration baseline</x:v>
       </x:c>
       <x:c r="F20" s="34" t="str">
-        <x:v>docs/testing/evidence/sprint-3/S3-EV-007-*</x:v>
+        <x:v>PR #78: https://github.com/JeraldBucud/GradNavi/pull/78 | PR #67: https://github.com/JeraldBucud/GradNavi/pull/67</x:v>
       </x:c>
       <x:c r="G20" s="34" t="str">
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="H20" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="I20" s="79" t="str"/>
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I20" s="84" t="n">
+        <x:v>46304</x:v>
+      </x:c>
       <x:c r="J20" s="34" t="str">
-        <x:v>Blocked until 6.3-6.7 ready</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
+        <x:v>WBS 6.5 merged to feature/sprint-3 through PR #59. Final WBS 6.7 integration occurred later through PR #78 on feature/sprint-4. Formal Sprint 3 closeout accepts the verified successor baseline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="54" customHeight="1">
       <x:c r="A21" s="34" t="str">
         <x:v>S3-EV-008</x:v>
       </x:c>
       <x:c r="B21" s="34" t="str">
-        <x:v>TBD</x:v>
+        <x:v>S3-TC-086:S3-TC-100</x:v>
       </x:c>
       <x:c r="C21" s="34" t="str">
         <x:v>6.9</x:v>
       </x:c>
       <x:c r="D21" s="34" t="str">
-        <x:v>Regression</x:v>
+        <x:v>Regression closeout</x:v>
       </x:c>
       <x:c r="E21" s="34" t="str">
-        <x:v>Sprint 3 final regression and quality evidence</x:v>
+        <x:v>Final backend, Django, migration, frontend, regression, browser/responsive/accessibility and evidence closeout accepted from verified successor testing</x:v>
       </x:c>
       <x:c r="F21" s="34" t="str">
-        <x:v>docs/testing/evidence/sprint-3/S3-EV-008-*</x:v>
+        <x:v>PR #74: https://github.com/JeraldBucud/GradNavi/pull/74 | PR #78: https://github.com/JeraldBucud/GradNavi/pull/78 | PR #67: https://github.com/JeraldBucud/GradNavi/pull/67 | docs/testing/sprint-4-test-cases.xlsx</x:v>
       </x:c>
       <x:c r="G21" s="34" t="str">
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="H21" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="I21" s="79" t="str"/>
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I21" s="84" t="n">
+        <x:v>46304</x:v>
+      </x:c>
       <x:c r="J21" s="34" t="str">
-        <x:v>Blocked until WBS 6.8 passes</x:v>
+        <x:v>Successor Sprint 4 verification finished with 129/129 planned cases Pass. Formal Sprint 3 evidence reconciliation is complete.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -6997,22 +7201,22 @@
       <x:c r="D23" t="str">
         <x:v>Screenshot</x:v>
       </x:c>
-      <x:c r="E23" t="str">
+      <x:c r="E23" s="34" t="str">
         <x:v>Shared feature/sprint-3 Django, migration, and Git baseline checks</x:v>
       </x:c>
-      <x:c r="F23" t="str">
+      <x:c r="F23" s="34" t="str">
         <x:v>docs/testing/evidence/sprint-3/S3-EV-009B-shared-backend-checks-and-status.png</x:v>
       </x:c>
-      <x:c r="G23" t="str">
+      <x:c r="G23" s="34" t="str">
         <x:v>Jerald</x:v>
       </x:c>
-      <x:c r="H23" t="str">
+      <x:c r="H23" s="34" t="str">
         <x:v>Captured</x:v>
       </x:c>
-      <x:c r="I23" s="80" t="n">
+      <x:c r="I23" s="79" t="n">
         <x:v>46278</x:v>
       </x:c>
-      <x:c r="J23" t="str">
+      <x:c r="J23" s="34" t="str">
         <x:v>Django system check passed; makemigrations --check reported no changes; feature/sprint-3 was up to date and working tree clean.</x:v>
       </x:c>
     </x:row>
@@ -7029,22 +7233,22 @@
       <x:c r="D24" t="str">
         <x:v>Screenshot</x:v>
       </x:c>
-      <x:c r="E24" t="str">
+      <x:c r="E24" s="34" t="str">
         <x:v>WBS 6.6 post-merge focused interview test suite</x:v>
       </x:c>
-      <x:c r="F24" t="str">
+      <x:c r="F24" s="34" t="str">
         <x:v>docs/testing/evidence/sprint-3/S3-EV-002F-wbs-6.6-post-merge-interview-tests.png</x:v>
       </x:c>
-      <x:c r="G24" t="str">
+      <x:c r="G24" s="34" t="str">
         <x:v>Jerald</x:v>
       </x:c>
-      <x:c r="H24" t="str">
+      <x:c r="H24" s="34" t="str">
         <x:v>Captured</x:v>
       </x:c>
-      <x:c r="I24" s="80" t="n">
+      <x:c r="I24" s="79" t="n">
         <x:v>46278</x:v>
       </x:c>
-      <x:c r="J24" t="str">
+      <x:c r="J24" s="34" t="str">
         <x:v>Fresh post-merge evidence: 38/38 interview tests passed in 9.057s; exit code 0.</x:v>
       </x:c>
     </x:row>
@@ -7060,7 +7264,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd7fbd3a6aeb49f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfdbc9da31ed48a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>